<commit_message>
Decide GAT Price structure: keep O&M in GATP, move only CLLC to capped Fuel Cost
After weighing all stakeholder comments, Sharon's and Antonette's
comments, DOE DC2026-06-0013 and the TOR: GATP = CRF + OM and
FC = FCC + CLLC. O&M returns to the GAT Price (DC 6.1(a); DC 4 and 7.2
define the FCPT as gas costs). Redline regenerated from the original
draft so it shows only the decided changes.

Also implement Antonette's comments 909 (ETA limited to mid-merit
intervals) and 918 (who pays non-mid-merit Fuel Cost energy), rebuild
the matrix addenda to match, conform the stale Section 11.5 remarks,
and add rules_decision_2026-10-19.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6VUATAmWPQdQ6XxJGJU7F
</commit_message>
<xml_diff>
--- a/GAIR_Comments_Matrix.xlsx
+++ b/GAIR_Comments_Matrix.xlsx
@@ -4189,7 +4189,7 @@
       <c r="F110" s="7" t="inlineStr">
         <is>
           <t>Adopted. ERC will include in the provisions clarifying this [Remark restored 24 Sep 2026 from the original ERC matrix, delete rows.xlsx.]
-[19 Oct 2026 update: See Row 143 as updated: the GAP now covers capital recovery only.]</t>
+[19 Oct 2026 update: See Row 143 as updated.]</t>
         </is>
       </c>
       <c r="G110" s="3" t="n"/>
@@ -4253,7 +4253,7 @@
       <c r="F113" s="7" t="inlineStr">
         <is>
           <t>Not adopted. GAT Price assumptions are fixed as a single Year-0 capital outlay solved on a levelized basis over the full Reference Operating Period (GAIR Sections 8.1, 8.3-8.4), and the resulting GAT Price/GAP is PHP-fixed under Section 8.5. The only permitted post-award adjustment is the one-time indexation under Section 11.5 between Certificate of Award and COD; no further indexation applies thereafter. This is consistent with DC2026-06-0013 Section 6.1's mandate that the GAT Price methodology balance ‘reasonable electricity rates for consumers while attracting sufficient investment’ (Sec. 6.1.3) — the levelization already prices in the expected life-of-project cost trajectory, and re-opening assumptions mid-term would shift risk back to consumers contrary to Section 8.5's policy. [Update 24 Sep 2026: the basis of each assumption must now be disclosed in the Reference Parameters Resolution (Section 8.7; Rules Comment 175).]
-[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 now covers only GAP adjustment for Lot 1 extensions, and Section 8.9 rules out any indexation of the GAT Price or GAP. The remark needs to be conformed to the current text.]</t>
+[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 covers only GAP adjustment for Lot 1 extensions, and Section 8.9 provides that the GAT Price and GAP are not indexed, escalated or adjusted for the term of the Certificate of Award. The disposition now rests on Section 8.9; any request for indexation is not adopted.]</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr">
@@ -4292,7 +4292,7 @@
       <c r="F114" s="7" t="inlineStr">
         <is>
           <t>Noted for clarification. Only the non-fuel GAT Price component is subject to competitive bidding (Section 5); Fuel Cost is excluded from bidding and recovered separately, capped at the Gas Price Benchmark (Sections 13-20), so a Winning Bidder's total rate can, in principle, exceed a rejected bidder's implied total rate if fuel costs differ — this is an inherent feature of separating capacity/non-fuel competition (price discovery) from a regulated, benchmarked Fuel Cost Pass-Through (cost containment), consistent with DC2026-06-0013 Section 8.2's 'full recovery of prudent and reasonable economic costs' principle. Consumer protection against excessive total cost is achieved not by comparing against non-Winning Bidders (who are not awarded and thus not comparable), but through the GAT Price ceiling (Section 5) on the competed component and the Gas Price Benchmark ceiling (Rule 3) and Section 25 audit on the pass-through component.
-[19 Oct 2026 update: Bids now compete on the capital recovery component only. The Fuel Cost now covers fuel commodity, logistics (CLLC) and O&amp;M (OMC), each capped uniformly for a Facility Type (Section 5 as revised).]</t>
+[19 Oct 2026 update: Bids now compete on capital recovery and O&amp;M. The Fuel Cost now covers the fuel commodity and logistics (CLLC), each capped uniformly for a Facility Type (Section 5 as revised).]</t>
         </is>
       </c>
       <c r="G114" s="3" t="inlineStr">
@@ -4545,7 +4545,7 @@
       <c r="F116" s="7" t="inlineStr">
         <is>
           <t>For Technical &amp; Legal Study in final GAIR determination.
-[19 Oct 2026 update: Status note: the draft Rules have moved the other way (GATP = CRF only; O&amp;M and logistics moved into the Fuel Cost). A fuel-inclusive GAT Price is not reflected in the draft; the final disposition should state the reasons.]</t>
+[19 Oct 2026 update: Not adopted. DC2026-06-0013 Section 7.2 and TOR Sections 4.2 and 17 pay the GAP and the Fuel Cost as separate components, and DC Section 4 defines the Fuel Cost Pass-Through separately, so a fuel-inclusive GAT Price would depart from the Circular. Competitive pressure on fuel is kept through the Gas Price Benchmark, the Section 17 caps, the Section 23 lesser-of certification and the savings-sharing provision.]</t>
         </is>
       </c>
       <c r="G116" s="3" t="inlineStr">
@@ -4582,10 +4582,9 @@
           <t>Comments/PMCJ Comments on Draft Rules - Gas Auction Threshold Price Determination Methodology.docx</t>
         </is>
       </c>
-      <c r="F117" s="7" t="inlineStr">
-        <is>
-          <t>Noted for clarification, and noted as to the broader policy argument (see the Commission's response on Section 2.5, above). On the specific question of duration: a consumer's payment obligation for a Winning Bidder's capital recovery, O&amp;M, G&amp;A, taxes, and equity return is not open-ended — it runs only for the Reference Operating Period fixed under Section 8.7 and Annex “A” Item A.8 (to be adopted consistent with the actual firm Certificate of Award term), after which the facility holds no automatic continuing entitlement to a GAT Price-based rate; further procurement from that facility beyond its awarded term requires participation in, and winning, a subsequent Auction Round under a newly solved GAT Price. Consumers are also protected during the award term by the FCPT audit/disallowance mechanism (Rule 4) and the annual Gas Price Benchmark review (Section 20), which prevent recovery of imprudent costs beyond the DCF Model's benchmarked parameters.
-[19 Oct 2026 update: O&amp;M and logistics costs are no longer in the GAT Price; they are passed through monthly as components of the Fuel Cost, each capped (Sections 17, 17-A) and audited (Section 25), with an annual O&amp;M true-up (Section 17-A.3).]</t>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>Noted for clarification, and noted as to the broader policy argument (see the Commission's response on Section 2.5, above). On the specific question of duration: a consumer's payment obligation for a Winning Bidder's capital recovery, O&amp;M, G&amp;A, taxes, and equity return is not open-ended — it runs only for the Reference Operating Period fixed under Section 8.7 and Annex “A” Item A.8 (to be adopted consistent with the actual firm Certificate of Award term), after which the facility holds no automatic continuing entitlement to a GAT Price-based rate; further procurement from that facility beyond its awarded term requires participation in, and winning, a subsequent Auction Round under a newly solved GAT Price. Consumers are also protected during the award term by the FCPT audit/disallowance mechanism (Rule 4) and the annual Gas Price Benchmark review (Section 20), which prevent recovery of imprudent costs beyond the DCF Model's benchmarked parameters.</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr">
@@ -5669,8 +5668,7 @@
       <c r="F142" s="7" t="inlineStr">
         <is>
           <t>Not adopted as proposed (annual CPI escalation); clarified. Per Section 8.3, the DCF Model's Annual Cash-Flow Projection uses the Fixed O&amp;M Costs, Variable Non-Fuel O&amp;M Costs, and G&amp;A Costs prescribed in Annex “A” as the Operating Expenditure input for every year of the Reference Operating Period; Section 8.3 does not itself provide, or contemplate, a separate year-by-year CPI/inflation escalation formula applied to these figures within the DCF projection. These Annex “A” reference values are fixed/constant in nominal PhP terms across the Reference Operating Period for purposes of the Section 8.4 iterative GAT Price solve, and are not further escalated year-by-year once the DCF Model is run. Expected inflation is instead already factored in once, at the point the reference O&amp;M and G&amp;A values are calculated and the GAT Price/GATP is solved: the Annex “A” Items A.4-A.6 Basis/Source references to re-basing historical PPA rates ‘to current price levels’ is that one-time calibration, distinct from — and not a substitute for — an ongoing annual escalator within the projection itself. This is consistent with Section 8.5 fixing the resulting GAT Price and GAP in PhP for the full term of the Certificate of Award, with the only further adjustment being the single, one-time Section 11.5 indexation between Certificate of Award and COD; no indexation applies for the remainder of the term. The Commission will make this fixed, non-CPI-escalated treatment of Annex “A” O&amp;M/G&amp;A values within the DCF projection explicit in the DCF Model's implementing computation guidelines ahead of the first Auction Round.
-[19 Oct 2026 update: Largely moot: Fixed and Variable O&amp;M are no longer DCF Operating Expenditure items. Actual O&amp;M is recovered through the Fuel Cost up to the O&amp;M Cost Caps, which are reviewed annually under Section 20, so cost escalation is reflected through the cap review rather than through escalation in the DCF. G&amp;A stays in the GAT Price.]
-[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 now covers only GAP adjustment for Lot 1 extensions, and Section 8.9 rules out any indexation of the GAT Price or GAP. The remark needs to be conformed to the current text.]</t>
+[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 covers only GAP adjustment for Lot 1 extensions, and Section 8.9 provides that the GAT Price and GAP are not indexed, escalated or adjusted for the term of the Certificate of Award. The disposition now rests on Section 8.9; any request for indexation is not adopted.]</t>
         </is>
       </c>
       <c r="G142" s="3" t="inlineStr">
@@ -5709,7 +5707,7 @@
       <c r="F143" s="7" t="inlineStr">
         <is>
           <t>Adopted with modification. The Commission will add an explanatory note/illustrative example to Rule 2 clarifying that the Gas Auction Price (GAP) endorsed to a Winning Bidder under DC2026-06-0013 Section 9.10-9.11 is the bidder's own winning Price Offer (which must not exceed the GAT Price ceiling per Section 5 and Circular Section 6.1), inclusive of the Capped Landed Logistics Cost the bidder priced into that offer under Section 8.6, subject to the Section 17/Annex A maximum caps. The GAP is therefore bidder-specific and market-determined at or below the GAT Price, not separately computed by the Commission; a worked numerical illustration will be added for clarity.
-[19 Oct 2026 update: The GAP is now the bidder's Price Offer for capital recovery only (CRF). The CLLC and O&amp;M are no longer part of the GAP; they are recovered through the Fuel Cost (Sections 8.6, 17-A, 18).]</t>
+[19 Oct 2026 update: The GAP is the bidder's Price Offer covering capital recovery and O&amp;M (CRF + OM). The CLLC is no longer part of the GAP; it is recovered through the Fuel Cost (Sections 8.6, 18).]</t>
         </is>
       </c>
       <c r="G143" s="3" t="inlineStr">
@@ -6801,7 +6799,7 @@
       <c r="F157" s="7" t="inlineStr">
         <is>
           <t>Not adopted. Section 8.5's fixed, PhP-denominated GAT Price/GAP for the full Certificate of Award term, and Section 11.5's single indexation window confined to the Award-to-COD gap, are deliberate risk-allocation choices, not oversights: extending indexation to post-COD macroeconomic shocks would reintroduce the same FX/inflation pass-through risk to consumers that Section 8.5 is designed to eliminate, and would undermine the price certainty that makes the GAT Price ceiling meaningful for competitive bidding. A Winning Bidder is expected to price its financing structure (currency mix, hedging, tenor) and the associated post-COD macro risk into its competitive Price Offer at the time of bidding, consistent with Section 2.5's cost-reflective, competitively-determined-price policy — macro risk borne after financial close is priced into the cost of capital ex ante under standard project-finance practice, not trued up ex post at consumers' expense.
-[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 now covers only GAP adjustment for Lot 1 extensions, and Section 8.9 rules out any indexation of the GAT Price or GAP. The remark needs to be conformed to the current text.]</t>
+[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 covers only GAP adjustment for Lot 1 extensions, and Section 8.9 provides that the GAT Price and GAP are not indexed, escalated or adjusted for the term of the Certificate of Award. The disposition now rests on Section 8.9; any request for indexation is not adopted.]</t>
         </is>
       </c>
       <c r="G157" s="3" t="inlineStr">
@@ -6971,7 +6969,7 @@
       <c r="F159" s="7" t="inlineStr">
         <is>
           <t>Adopted with modification. Section 8.6 embeds the Capped Landed Logistics Cost as a levelized Operating Expenditure item precisely so that ‘the Winning Bidder, and not the electricity consumer, bears the risk of gas-delivery-infrastructure underutilization’ — this is Section 8.6's express policy, not an oversight. However, the Commission agrees that where actual dispatch is materially below the Reference Net Capacity Factor (Annex “A” Item A.2) for reasons outside the Winning Bidder's control (e.g., System-Operator-directed curtailment per Section 28(h)), an adjustment may be warranted. The Commission will address this through the Section 28(h) treatment of curtailment (see Comment No. 15) rather than by reopening Section 8.6/13.4's fixed, capped-and-embedded CLLC design, to avoid reintroducing the logistics-cost volatility Section 8.6 is designed to shield consumers from.
-[19 Oct 2026 update: The rationale above (Winning Bidder bears underutilization risk inside the GAT Price) no longer applies: the CLLC is now recovered through the Fuel Cost per MMBtu burned, up to the Section 17 caps. Tokyo Gas's specific point is still open, because fixed terminal-capacity and pipeline reservation charges are recovered only on gas actually burned and so are still under-recovered when dispatch is below the Reference Net Capacity Factor. For Commission decision.]</t>
+[19 Oct 2026 update: Rationale above superseded: the CLLC is now recovered through the Fuel Cost per MMBtu burned, up to the Section 17 caps. Not adopted as to capacity-based recovery of fixed terminal-capacity and pipeline reservation charges: Section 28 and TOR Sections 4.2 and 17 pay only per kWh delivered. The caps are set per MMBtu at the Reference Net Capacity Factor, so the Winning Bidder carries the volume risk when dispatch is lower.]</t>
         </is>
       </c>
       <c r="G159" s="3" t="inlineStr">
@@ -7020,7 +7018,7 @@
       <c r="F160" s="7" t="inlineStr">
         <is>
           <t>Adopted with modification. The Section 17/Annex “A” Item A.17 caps (regasification/terminal, pipeline transportation, BOG loss) are default uniform ceilings per DC2026-06-0013 Section 18.2.2, but Section 17 already allows a Winning Bidder to demonstrate higher prudent, project-specific costs subject to Commission approval. The Commission adopts the recommended ‘benchmark-plus-project-specific review’ framing: Section 17 will be amended (together with the review-timeline amendment in Comment No. 11) to expressly permit differentiation based on terminal, geographic location, contractual arrangement, infrastructure configuration, and gas-delivery route, supported by executed terminal/pipeline agreements and competitive quotations, while Section 20's annual review continues to update the standard default caps. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.] [Implemented 24 Sep 2026: Section 17's above-cap evaluation criteria now list terminal, location, contractual arrangement, infrastructure configuration and delivery route, supported by executed agreements (Rules Comment 179).]
-[19 Oct 2026 update: Caps may now be set separately for each Fuel Source Category (Section 17), and they now limit the CLLC component of the Fuel Cost rather than a GAT Price allowance.]</t>
+[19 Oct 2026 update: Caps may now be set separately for each Fuel Source Category (Section 17), and they now limit the CLLC component of the Fuel Cost instead of a GAT Price allowance.]</t>
         </is>
       </c>
       <c r="G160" s="3" t="inlineStr">
@@ -7059,8 +7057,8 @@
       <c r="F161" s="7" t="inlineStr">
         <is>
           <t>Adopted with modification. CLLC is fixed for the delivery period once embedded in the bidder's winning GAP under Section 8.6 (subject only to the Section 11.5 one-time indexation) — it is not subsequently trued up to actual logistics costs, consistent with Section 8.6's policy that the Winning Bidder bears logistics-cost/underutilization risk. The Section 17 exception for above-cap costs applies only prospectively, to costs the bidder could not have foreseen and priced into its offer, upon Commission approval. The Commission adopts MERALCO's proposal that, where bidders submit CLLC values as part of their offer, the Allowable Add-On Cost Caps used to police the offer shall be the lower of the Commission's maximum cap under Section 17/Annex A Item A.17 and the CLLC value submitted by the bidder, and will revise Section 17 accordingly. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.]
-[19 Oct 2026 update: The first part of this disposition no longer holds: the draft Rules now set GATP = CRF (capital recovery only) and move the Capped Landed Logistics Cost (CLLC) and fixed/variable O&amp;M (OMC) into the Fuel Cost, FC = FCC + CLLC + OMC, each component at the lesser of actual prudent cost and a maximum cap (Sections 8.6, 13.4, 17, new 17-A, 18). The CLLC is no longer fixed inside the GAP; it is billed monthly at the lesser of actual cost and cap. The lower-of rule for a bidder-disclosed CLLC value is kept in Section 17.]
-[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 now covers only GAP adjustment for Lot 1 extensions, and Section 8.9 rules out any indexation of the GAT Price or GAP. The remark needs to be conformed to the current text.]</t>
+[19 Oct 2026 update: The first part of this disposition no longer holds. Decision of 19 Oct 2026: the GAT Price stays CRF + OM, and the Capped Landed Logistics Cost (CLLC) moves out of the GAT Price into the Fuel Cost as a capped component, FC = FCC + CLLC, each add-on component at the lesser of actual prudent cost and its Section 17 cap (Sections 8.6, 13.4, 17, 18). The CLLC is no longer fixed inside the GAP; it is billed monthly at the lesser of actual cost and cap. The adopted lower-of rule for a bidder-disclosed CLLC value is kept in Section 17.]
+[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 covers only GAP adjustment for Lot 1 extensions, and Section 8.9 provides that the GAT Price and GAP are not indexed, escalated or adjusted for the term of the Certificate of Award. The disposition now rests on Section 8.9; any request for indexation is not adopted.]</t>
         </is>
       </c>
       <c r="G161" s="3" t="inlineStr">
@@ -7097,7 +7095,7 @@
       <c r="F162" s="7" t="inlineStr">
         <is>
           <t>Not adopted; same disposition as the Commission’s response to the related comment on this Section above. Section 8.6’s embedding of the Capped Landed Logistics Cost as a levelized, capped Operating Expenditure item — rather than a pass-through recovered dollar-for-dollar under Rule 4 — is a deliberate risk-allocation choice, not an oversight: it caps consumers’ exposure to logistics-cost overruns and shifts that risk to the Winning Bidder, consistent with DC2026-06-0013 Section 18.2.2’s mandate to impose "strict limitations and price caps on allowable add-on costs...to prevent the passing of unwarranted fuel procurement costs to consumers." Converting CLLC to an uncapped, audit-based FCPT item, as Aboitiz proposes here (and again for Section 13.4 below), would reintroduce the very cost-pass-through volatility Section 8.6 is designed to prevent. The Commission notes Section 17 already provides a facility-specific escape valve for above-cap costs, upon a documented showing of prudence and unavoidability. [Remark restored 24 Sep 2026 from the original ERC matrix, delete rows.xlsx.]
-[19 Oct 2026 update: Superseded; now adopted in part. The draft Rules now set GATP = CRF (capital recovery only) and move the Capped Landed Logistics Cost (CLLC) and fixed/variable O&amp;M (OMC) into the Fuel Cost, FC = FCC + CLLC + OMC, each component at the lesser of actual prudent cost and a maximum cap (Sections 8.6, 13.4, 17, new 17-A, 18). Aboitiz's request to recover actual landed logistics costs through the FCPT is therefore adopted. Its request to drop the caps is still not adopted: each add-on component stays capped under Section 17, consistent with DC2026-06-0013 Section 18.2.2. See the 19 Oct 2026 comment on Section 8.6 in the draft Rules.]</t>
+[19 Oct 2026 update: Superseded; now adopted in part. Decision of 19 Oct 2026: the GAT Price stays CRF + OM, and the Capped Landed Logistics Cost (CLLC) moves out of the GAT Price into the Fuel Cost as a capped component, FC = FCC + CLLC, each add-on component at the lesser of actual prudent cost and its Section 17 cap (Sections 8.6, 13.4, 17, 18). Aboitiz's request to recover actual landed logistics costs through the FCPT is adopted. Its request to drop the caps is still not adopted: each add-on component stays capped under Section 17, as DC2026-06-0013 Section 18.2.2 requires.]</t>
         </is>
       </c>
       <c r="G162" s="3" t="n"/>
@@ -8312,7 +8310,7 @@
       <c r="F196" s="7" t="inlineStr">
         <is>
           <t>Adopted. Where the Commission determines separate GAT Price determinations are warranted for technology sub-categories under Section 10 (e.g., FSRU-based Imported LNG versus pipeline-based Indigenous gas, where infrastructure type materially affects non-fuel project costs), all applicable GAT Prices for the relevant Auction Round shall be made known and available to all Bidders concurrently, consistent with the Commission’s obligation under Section 7 to issue GAT Prices for "each applicable Facility Type" within the prescribed timeline, and to avoid any risk of an uneven or sequential disclosure distorting the ranking of Price Offers. [Remark restored 24 Sep 2026 from the original ERC matrix, delete rows.xlsx.]
-[19 Oct 2026 update: With logistics costs out of the GAT Price, any separate GAT Price for technology sub-categories under Section 10 would rest on capital-cost differences only.]</t>
+[19 Oct 2026 update: With logistics costs out of the GAT Price, any separate GAT Price for technology sub-categories under Section 10 would rest on capital and O&amp;M cost differences only.]</t>
         </is>
       </c>
       <c r="G196" s="3" t="n"/>
@@ -8571,7 +8569,7 @@
       <c r="F205" s="7" t="inlineStr">
         <is>
           <t>Not adopted. Section 11.5's one-time indexation between Certificate of Award and COD, with no further indexation thereafter, mirrors the Commission's existing practice under the DOE's Green Energy Auction Program (GEAP) referenced in that Section, and is a deliberate risk allocation: it fixes non-fuel cost risk on the Winning Bidder for the remainder of the term (consistent with Section 8.5's PHP-Denominated Settlement policy) so that only genuinely volatile Fuel Costs are trued up periodically (Sections 20 and 23). Winning Bidders price this risk into their non-fuel Price Offer at bid stage under DC2026-06-0013 Section 8.2 ('full recovery of prudent and reasonable economic costs...provided that the Winning Bidder's price offer reflects such prudent and reasonable costs').
-[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 now covers only GAP adjustment for Lot 1 extensions, and Section 8.9 rules out any indexation of the GAT Price or GAP. The remark needs to be conformed to the current text.]</t>
+[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 covers only GAP adjustment for Lot 1 extensions, and Section 8.9 provides that the GAT Price and GAP are not indexed, escalated or adjusted for the term of the Certificate of Award. The disposition now rests on Section 8.9; any request for indexation is not adopted.]</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr">
@@ -8611,7 +8609,7 @@
       <c r="F206" s="7" t="inlineStr">
         <is>
           <t>Not adopted (scope); Adopted (mechanics disclosure). The one-time indexation properly applies to both the GAT Price and the corresponding endorsed GAP because the GAT Price is the ceiling from which the GAP is derived (Section 5) — indexing only the GAP without adjusting the underlying ceiling could allow a GAP that no longer reflects the Section 8 DCF Model's updated cost benchmarks to exceed a stale GAT Price, or conversely trap a prudent adjustment against an un-indexed ceiling. The rationale (Section 11.5) is to reconcile the DCF Model's Year-0 cost assumptions (Annex A) with verified movements in cost benchmarks between Certificate of Award and COD, consistent with the Commission's GEAP indexation practice. The Commission adopts MERALCO's request to detail the implementing mechanism (data sources, verification steps, and computation) for the one-time indexation adjustment as a new Section 11.6 or Annex provision.
-[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 now covers only GAP adjustment for Lot 1 extensions, and Section 8.9 rules out any indexation of the GAT Price or GAP. The remark needs to be conformed to the current text.]</t>
+[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 covers only GAP adjustment for Lot 1 extensions, and Section 8.9 provides that the GAT Price and GAP are not indexed, escalated or adjusted for the term of the Certificate of Award. The disposition now rests on Section 8.9; any request for indexation is not adopted.]</t>
         </is>
       </c>
       <c r="G206" s="3" t="inlineStr">
@@ -10263,10 +10261,9 @@
           <t>Comments/Annex B - SPPC and EERI Comments on Gas Auction Implementing Rules.docx</t>
         </is>
       </c>
-      <c r="F245" s="7" t="inlineStr">
-        <is>
-          <t>Adopted with modification. The Commission will publish the initial default caps for each add-on cost component (regasification/terminal, pipeline transportation, BOG loss allowance) concurrently with the first GAT Price issuance under Section 7.1, consistent with DC2026-06-0013 Section 18.2.2's mandate that the ERC ‘establish and publish a Gas Price Benchmarking methodology...defin[ing]...strict limitations or price caps on add-on costs.’ Reference default values are provided in mid_merit_gas_rates.xlsx, ‘Fuel Benchmarking &amp; Audit’ sheet (Regas/Terminal cap USD1.20/MMBtu; Pipeline cap USD0.80/MMBtu; BOG loss 0.50%). Section 17 will be amended to clarify that the ‘three (3) comparable third-party service quotations’ default applies at Supply Agreement execution and is not automatically re-triggered by routine monthly FCPT adjustments, which instead apply the then-current Commission-approved cap. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.] [24 Sep 2026 note: the cap and heat-rate figures cited in this remark come from mid_merit_gas_rates.xlsx (e.g., USD1.20/MMBtu regasification, USD0.80/MMBtu pipeline, 0.50% BOG; 7,200/10,000/8,500 Btu/kWh). They differ from the claudenumbers working file (USD1.50/MMBtu; BOG 0.10%/day; 6,100/6,350/9,800/8,000 Btu/kWh). Neither set has an identified external source. Values will be fixed in the Reference Parameters Resolution, not in the Rules; see Rules Comments 164–165.]
-[19 Oct 2026 update: The O&amp;M Cost Caps under new Section 17-A are also to be published together with the GAT Price.]</t>
+      <c r="F245" s="3" t="inlineStr">
+        <is>
+          <t>Adopted with modification. The Commission will publish the initial default caps for each add-on cost component (regasification/terminal, pipeline transportation, BOG loss allowance) concurrently with the first GAT Price issuance under Section 7.1, consistent with DC2026-06-0013 Section 18.2.2's mandate that the ERC ‘establish and publish a Gas Price Benchmarking methodology...defin[ing]...strict limitations or price caps on add-on costs.’ Reference default values are provided in mid_merit_gas_rates.xlsx, ‘Fuel Benchmarking &amp; Audit’ sheet (Regas/Terminal cap USD1.20/MMBtu; Pipeline cap USD0.80/MMBtu; BOG loss 0.50%). Section 17 will be amended to clarify that the ‘three (3) comparable third-party service quotations’ default applies at Supply Agreement execution and is not automatically re-triggered by routine monthly FCPT adjustments, which instead apply the then-current Commission-approved cap. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.] [24 Sep 2026 note: the cap and heat-rate figures cited in this remark come from mid_merit_gas_rates.xlsx (e.g., USD1.20/MMBtu regasification, USD0.80/MMBtu pipeline, 0.50% BOG; 7,200/10,000/8,500 Btu/kWh). They differ from the claudenumbers working file (USD1.50/MMBtu; BOG 0.10%/day; 6,100/6,350/9,800/8,000 Btu/kWh). Neither set has an identified external source. Values will be fixed in the Reference Parameters Resolution, not in the Rules; see Rules Comments 164–165.]</t>
         </is>
       </c>
       <c r="G245" s="3" t="inlineStr">
@@ -10309,7 +10306,7 @@
       <c r="F246" s="7" t="inlineStr">
         <is>
           <t>Adopted. Section 17 will be amended to clarify that a Winning Bidder's own dedicated regasification facility, if capitalized as part of the project (rather than procured under a third-party service agreement), is properly includible in the All-In Project Cost under Section 8.1 and recovered at the project's WACC (Section 8.2), subject to the Section 11.5 true-up, and that the Allowable Add-On Cost Caps under Section 17 apply only to genuine third-party regasification/terminal service agreements — consistent with Section 17's existing anti-double-recovery rule that no cost may be counted in both the GAT Price components and the Allowable Add-On Costs, verified under the Section 25 audit. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.]
-[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 now covers only GAP adjustment for Lot 1 extensions, and Section 8.9 rules out any indexation of the GAT Price or GAP. The remark needs to be conformed to the current text.]</t>
+[19 Oct 2026 update: this remark relies on a "Section 11.5" one-time indexation between Certificate of Award and COD. The current draft Rules have no such provision: Section 11 covers only GAP adjustment for Lot 1 extensions, and Section 8.9 provides that the GAT Price and GAP are not indexed, escalated or adjusted for the term of the Certificate of Award. The disposition now rests on Section 8.9; any request for indexation is not adopted.]</t>
         </is>
       </c>
       <c r="G246" s="3" t="inlineStr">
@@ -10418,10 +10415,9 @@
           <t>Comments/PEI and SEDI comments_draft ERC Reso(GAT Price) Case no. 2026-015 RM.pdf [OCR-transcribed from scanned PDF]</t>
         </is>
       </c>
-      <c r="F249" s="7" t="inlineStr">
-        <is>
-          <t>Adopted; same disposition as Comment No. 9. The Commission will publish the initial default add-on cost caps concurrently with the first GAT Price issuance under Section 7.1 (no later than sixty (60) calendar days after ITB issuance for the first Auction Round, per DC2026-06-0013 Section 6.1's parallel first-round timeline; DC2026-06-0013 Section 9.3 separately gives the DOE thirty (30) calendar days after the ERC's issuance to publish it), using the methodology and reference values in mid_merit_gas_rates.xlsx, ‘Fuel Benchmarking &amp; Audit’ sheet (Regas/Terminal cap USD1.20/MMBtu; Pipeline cap USD0.80/MMBtu; BOG loss 0.50%) as the Commission's working reference basis, subject to Section 20's annual review. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.] [24 Sep 2026 note: the cap and heat-rate figures cited in this remark come from mid_merit_gas_rates.xlsx (e.g., USD1.20/MMBtu regasification, USD0.80/MMBtu pipeline, 0.50% BOG; 7,200/10,000/8,500 Btu/kWh). They differ from the claudenumbers working file (USD1.50/MMBtu; BOG 0.10%/day; 6,100/6,350/9,800/8,000 Btu/kWh). Neither set has an identified external source. Values will be fixed in the Reference Parameters Resolution, not in the Rules; see Rules Comments 164–165.]
-[19 Oct 2026 update: See Row 245 as updated.]</t>
+      <c r="F249" s="3" t="inlineStr">
+        <is>
+          <t>Adopted; same disposition as Comment No. 9. The Commission will publish the initial default add-on cost caps concurrently with the first GAT Price issuance under Section 7.1 (no later than sixty (60) calendar days after ITB issuance for the first Auction Round, per DC2026-06-0013 Section 6.1's parallel first-round timeline; DC2026-06-0013 Section 9.3 separately gives the DOE thirty (30) calendar days after the ERC's issuance to publish it), using the methodology and reference values in mid_merit_gas_rates.xlsx, ‘Fuel Benchmarking &amp; Audit’ sheet (Regas/Terminal cap USD1.20/MMBtu; Pipeline cap USD0.80/MMBtu; BOG loss 0.50%) as the Commission's working reference basis, subject to Section 20's annual review. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.] [24 Sep 2026 note: the cap and heat-rate figures cited in this remark come from mid_merit_gas_rates.xlsx (e.g., USD1.20/MMBtu regasification, USD0.80/MMBtu pipeline, 0.50% BOG; 7,200/10,000/8,500 Btu/kWh). They differ from the claudenumbers working file (USD1.50/MMBtu; BOG 0.10%/day; 6,100/6,350/9,800/8,000 Btu/kWh). Neither set has an identified external source. Values will be fixed in the Reference Parameters Resolution, not in the Rules; see Rules Comments 164–165.]</t>
         </is>
       </c>
       <c r="G249" s="3" t="inlineStr">
@@ -10462,7 +10458,7 @@
       <c r="F250" s="7" t="inlineStr">
         <is>
           <t>Not adopted as to the add-on cost caps being undetermined and bidder-set by default; noted as to the climate/methane policy argument (addressed in the Commission's response on Section 2.5). On the caps: Section 17 does not leave consumers unprotected pending the Commission's determination of specific numeric caps — the default fallback is “the most recent Commission-approved or DOE-regulated tariff or rate for the corresponding service,” and only “in the absence thereof” may a Winning Bidder submit an average of at least three (3) comparable third-party service quotations, which remain “subject to Commission verification” before being accepted as the interim cap; a bidder cannot unilaterally fix its own ceiling. The Commission must likewise review and update the specific numeric caps under Section 20, and no cost recovered as an Allowable Add-On Cost may simultaneously be embedded in Fixed O&amp;M, Variable O&amp;M, G&amp;A, or All-In Project Cost, with the absence of such double recovery independently verified in the Section 25 audit. The Commission will prioritize finalizing specific numeric caps for each add-on cost component ahead of the first Auction Round, to reduce reliance on the bidder-quotation fallback. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.]
-[19 Oct 2026 update: The caps now limit pass-through amounts: logistics and O&amp;M costs are recovered through the Fuel Cost at the lesser of actual prudent cost and the Section 17/17-A caps, so consumers now bear changes in these costs up to the caps.]</t>
+[19 Oct 2026 update: The caps now limit pass-through amounts: logistics costs are recovered through the Fuel Cost at the lesser of actual prudent cost and the Section 17 caps.]</t>
         </is>
       </c>
       <c r="G250" s="3" t="inlineStr">
@@ -11005,7 +11001,7 @@
       <c r="F269" s="7" t="inlineStr">
         <is>
           <t>Adopted. Section 18(d) is revised to expressly include Republic Act No. 12120 (Philippine Natural Gas Industry Development Act) alongside the existing Republic Act No. 11534 (CREATE Act) and PEZA references, so that any VAT exemption or zero-rating available to logistics costs embedded in the GAT Price under RA 12120 is likewise excluded from the GAT Price to the extent of such exemption, subject to Commission verification. On the broader point that RA 12120's VAT exemption extends to total power generated and not solely the Fuel Cost component: noted for the Commission's separate evaluation of how RA 12120 fiscal incentives interact with the non-fuel GAT Price and DCF Model parameters (Annex “A” Item A.14), which may be addressed in a future clarificatory issuance, since Section 18(d) itself is confined to the Fuel VAT Rate used in the FCPT computation. [24 Sep 2026 correction: an annotation citing a “forensic audit” of named plants (terminal charges of USD2.93/MMBtu, a USD15.66M “disallowance precedent”, a “SIGTTO/DNV” BOG limit and a 0.88 JKM regression) has been removed. USD2.93/MMBtu is the White Paper's modelled logistics cost (Clarete 2018, CPI-inflated), not a billed fee. No Commission finding supports the other figures. See Rules Comment 164.]
-[19 Oct 2026 update: See Row 263 as updated: the exemption now operates on the CLLC component of the Fuel Cost.]</t>
+[19 Oct 2026 update: See Row 263 as updated: the exemption now applies to the CLLC component of the Fuel Cost.]</t>
         </is>
       </c>
       <c r="G269" s="3" t="inlineStr">
@@ -15227,10 +15223,9 @@
           <t>Comments/Public Consultation_ERC CASE NO. 2026-015 RM_Siemens Energy Comments.pdf</t>
         </is>
       </c>
-      <c r="F415" s="7" t="inlineStr">
-        <is>
-          <t>Noted for clarification. The Fixed and Variable O&amp;M reference values under Annex “A” Items A.4-A.5 are sourced, per Annex “A”'s own stated Basis/Source, from the FGP San Lorenzo PPA (Article 5, Sections 5.2(b)-(e)), re-based to current price levels. The Commission acknowledges actual O&amp;M costs vary by OEM, maintenance contract structure, and plant configuration; however, since a single reference project is used to solve one levelized GAT Price per Facility Type under Section 8.1, the Commission's approach adopts one contractually-documented reference O&amp;M benchmark rather than a facility-specific figure for each prospective bidder's differing OEM or maintenance arrangement. A Winning Bidder's own actual O&amp;M cost structure does not separately enter into GAT Price or FCPT computation, since Fixed and Variable O&amp;M is embedded in the non-fuel GAT Price ceiling determined competitively through the Auction. [Update 24 Sep 2026: O&amp;M benchmark basis must be disclosed under Section 8.7 (Rules Comment 175).]
-[19 Oct 2026 update: The Annex "A" Items A.4-A.5 values now set the O&amp;M Cost Caps under Section 17-A; they are no longer DCF Operating Expenditure inputs (except where G&amp;A is computed as a percentage of O&amp;M).]</t>
+      <c r="F415" s="3" t="inlineStr">
+        <is>
+          <t>Noted for clarification. The Fixed and Variable O&amp;M reference values under Annex “A” Items A.4-A.5 are sourced, per Annex “A”'s own stated Basis/Source, from the FGP San Lorenzo PPA (Article 5, Sections 5.2(b)-(e)), re-based to current price levels. The Commission acknowledges actual O&amp;M costs vary by OEM, maintenance contract structure, and plant configuration; however, since a single reference project is used to solve one levelized GAT Price per Facility Type under Section 8.1, the Commission's approach adopts one contractually-documented reference O&amp;M benchmark rather than a facility-specific figure for each prospective bidder's differing OEM or maintenance arrangement. A Winning Bidder's own actual O&amp;M cost structure does not separately enter into GAT Price or FCPT computation, since Fixed and Variable O&amp;M is embedded in the non-fuel GAT Price ceiling determined competitively through the Auction. [Update 24 Sep 2026: O&amp;M benchmark basis must be disclosed under Section 8.7 (Rules Comment 175).]</t>
         </is>
       </c>
       <c r="G415" s="3" t="inlineStr">
@@ -15258,10 +15253,9 @@
       </c>
       <c r="D416" s="3" t="n"/>
       <c r="E416" s="3" t="n"/>
-      <c r="F416" s="7" t="inlineStr">
-        <is>
-          <t>Noted. O&amp;M reference values will be fixed and updated before each Auction Round in the Reference Parameters Resolution, with sources disclosed under Section 8.7 (Rules Comment 175). Candidate values are recorded in Rules Comment 162.
-[19 Oct 2026 update: See Row 415 as updated.]</t>
+      <c r="F416" s="3" t="inlineStr">
+        <is>
+          <t>Noted. O&amp;M reference values will be fixed and updated before each Auction Round in the Reference Parameters Resolution, with sources disclosed under Section 8.7 (Rules Comment 175). Candidate values are recorded in Rules Comment 162.</t>
         </is>
       </c>
       <c r="G416" s="3" t="n"/>
@@ -15341,10 +15335,9 @@
           <t>Comments/PCG_Consolidated Comments_20260814 [Clean].pdf</t>
         </is>
       </c>
-      <c r="F418" s="7" t="inlineStr">
-        <is>
-          <t>Adopted for further Commission study. Annex “A” Item A.6 currently sets the G&amp;A percentage itself as “to be determined by the Commission,” with the stated basis described only as “General ERC rate-case practice (a range of combined O&amp;M); midpoint to be determined.” The Commission agrees this basis should be made independently verifiable before a final G&amp;A figure is adopted, whether by disclosing the specific historical ERC rate cases and range relied upon, or by benchmarking G&amp;A against the actual G&amp;A run-rate of comparable existing mid-merit gas plants already referenced elsewhere in Annex “A” for other parameters (e.g., the Item A.1 peer mid-merit fleet capacities and the Item A.3 CAPEX benchmark plants), to the extent such G&amp;A-specific data can be independently documented. The Commission will disclose its supporting rate-case basis and computation when Item A.6 is finalized, in the interest of transparency and to allow stakeholders to verify the reasonableness of the adopted G&amp;A figure before the first Auction Round. [Update 24 Sep 2026: the 7.5% G&amp;A formula was removed from Annex “A” (Rules Comments 111 and 139); the G&amp;A basis must be disclosed under Section 8.7 (Rules Comment 175).]
-[19 Oct 2026 update: G&amp;A remains in the GAT Price. Where G&amp;A is expressed as a percentage of O&amp;M, the Items A.4-A.5 reference values are still used for that calculation.]</t>
+      <c r="F418" s="3" t="inlineStr">
+        <is>
+          <t>Adopted for further Commission study. Annex “A” Item A.6 currently sets the G&amp;A percentage itself as “to be determined by the Commission,” with the stated basis described only as “General ERC rate-case practice (a range of combined O&amp;M); midpoint to be determined.” The Commission agrees this basis should be made independently verifiable before a final G&amp;A figure is adopted, whether by disclosing the specific historical ERC rate cases and range relied upon, or by benchmarking G&amp;A against the actual G&amp;A run-rate of comparable existing mid-merit gas plants already referenced elsewhere in Annex “A” for other parameters (e.g., the Item A.1 peer mid-merit fleet capacities and the Item A.3 CAPEX benchmark plants), to the extent such G&amp;A-specific data can be independently documented. The Commission will disclose its supporting rate-case basis and computation when Item A.6 is finalized, in the interest of transparency and to allow stakeholders to verify the reasonableness of the adopted G&amp;A figure before the first Auction Round. [Update 24 Sep 2026: the 7.5% G&amp;A formula was removed from Annex “A” (Rules Comments 111 and 139); the G&amp;A basis must be disclosed under Section 8.7 (Rules Comment 175).]</t>
         </is>
       </c>
       <c r="G418" s="3" t="inlineStr">
@@ -18029,7 +18022,7 @@
       <c r="F566" s="7" t="inlineStr">
         <is>
           <t>For Technical &amp; Legal Study in final GAIR determination.
-[19 Oct 2026 update: See Row 116 status note.]</t>
+[19 Oct 2026 update: Not adopted; see Row 116.]</t>
         </is>
       </c>
       <c r="G566" s="3" t="inlineStr">
@@ -19059,7 +19052,7 @@
       <c r="F574" s="7" t="inlineStr">
         <is>
           <t>For Technical &amp; Legal Study in final GAIR determination.
-[19 Oct 2026 update: Pipeline transportation costs are no longer incorporated into the GAT Price; they are recovered through the CLLC component of the Fuel Cost, capped under Section 17.]</t>
+[19 Oct 2026 update: Pipeline transportation costs are no longer in the GAT Price; they are recovered through the CLLC component of the Fuel Cost, capped under Section 17.]</t>
         </is>
       </c>
       <c r="G574" s="3" t="inlineStr">
@@ -19962,7 +19955,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Rows 116, 566, 574 updated: draft now moves O&amp;M and logistics out of the GAT Price, the opposite of the fuel-inclusive GAT proposal.</t>
+          <t>Rows 116 and 566 (fuel-inclusive GAT Price) decided: not adopted. Row 574 updated.</t>
         </is>
       </c>
     </row>
@@ -20070,11 +20063,6 @@
           <t>54, 175, 176</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Row 415 updated: O&amp;M values now set the Section 17-A caps.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
@@ -20110,11 +20098,6 @@
           <t>14, 23, 29, 33, 41, 75, 86, 177</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>Row 249 updated (O&amp;M caps published with GAT Price).</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
@@ -20152,7 +20135,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Rows 110, 114, 143, 161, 263 updated for the GATP = CRF restructure; Row 161 (CLLC fixed in GAP) no longer holds.</t>
+          <t>Rows 110, 114, 143, 161, 263 updated for the 19 Oct decision (CLLC moved to the FC; GAT Price = CRF + OM). Row 161 (CLLC fixed in GAP) superseded.</t>
         </is>
       </c>
     </row>
@@ -20192,7 +20175,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Rows 159, 160 updated. Fixed terminal/pipeline charges under low dispatch remain open (Row 159).</t>
+          <t>Rows 159, 160 updated; capacity-based recovery of fixed logistics charges not adopted (Row 159).</t>
         </is>
       </c>
     </row>
@@ -20337,7 +20320,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Rows 142, 217, 245 updated (O&amp;M escalation largely moot; add-on costs now via FCPT).</t>
+          <t>Row 217 updated (add-on costs now via the FCPT).</t>
         </is>
       </c>
     </row>
@@ -20377,7 +20360,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Rows 117, 250 updated: O&amp;M and logistics now passed through up to caps.</t>
+          <t>Row 250 updated: caps now limit logistics pass-through.</t>
         </is>
       </c>
     </row>
@@ -20417,7 +20400,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Rows 269, 418 updated.</t>
+          <t>Row 269 updated.</t>
         </is>
       </c>
     </row>
@@ -20494,7 +20477,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Rows 162, 218 (logistics through FCPT instead of GAT Price) now adopted in part; caps retained (Rows 251, 254-262, 297).</t>
+          <t>Rows 162, 218 (logistics through the FCPT instead of the GAT Price) now adopted in part; caps retained (Rows 251, 254-262, 297).</t>
         </is>
       </c>
     </row>

</xml_diff>